<commit_message>
Final README, golden-50 evaluation and error analysis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labeling/golden_50_labeling.xlsx
+++ b/labeling/golden_50_labeling.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/laurabernal/Documents/Claude/Multi Agent Pipeline/labeling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAB832D-E9A4-4148-BFBF-A96269062070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6859DE-D687-5D43-A43A-4F8AD64B1E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="191">
   <si>
     <t>#</t>
   </si>
@@ -570,6 +570,48 @@
   </si>
   <si>
     <t>0.5</t>
+  </si>
+  <si>
+    <t>-0.5</t>
+  </si>
+  <si>
+    <t>Cant recognize the language</t>
+  </si>
+  <si>
+    <t>ads</t>
+  </si>
+  <si>
+    <t>shuffle, premium</t>
+  </si>
+  <si>
+    <t>lyrics, update</t>
+  </si>
+  <si>
+    <t>update, rewind</t>
+  </si>
+  <si>
+    <t>update</t>
+  </si>
+  <si>
+    <t>wen I play my song it o ly plays a little bit then it stops</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> it keeps crashing every time. </t>
+  </si>
+  <si>
+    <t>I was able to put in only a few songs I like and Spotify gave me recommendations</t>
+  </si>
+  <si>
+    <t>we cannot playback the songs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">we can't choose our fvrt songs after some clicks, we can't CHOOSE song after a song played, and we can't turn off shuffle option. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">I'm trying to play a song but it doesn't working. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">suddenly an add starts and my ears feel like they explode!! </t>
   </si>
 </sst>
 </file>
@@ -659,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -679,6 +721,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -981,7 +1026,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1041,7 +1085,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1051,16 +1095,22 @@
       <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="3"/>
+      <c r="D2" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E2" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3">
+        <v>2</v>
+      </c>
       <c r="G2" s="3">
         <v>-1</v>
       </c>
       <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
@@ -1068,7 +1118,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1078,11 +1128,15 @@
       <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E3" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F3" s="3"/>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
       <c r="G3" s="3">
         <v>1</v>
       </c>
@@ -1095,7 +1149,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1105,11 +1159,15 @@
       <c r="C4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3"/>
+      <c r="D4" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E4" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F4" s="3"/>
+      <c r="F4" s="3">
+        <v>1</v>
+      </c>
       <c r="G4" s="3">
         <v>1</v>
       </c>
@@ -1132,12 +1190,22 @@
       <c r="C5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F5" s="3">
+        <v>2</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
@@ -1145,7 +1213,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1155,11 +1223,15 @@
       <c r="C6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E6" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F6" s="3"/>
+      <c r="F6" s="3">
+        <v>1</v>
+      </c>
       <c r="G6" s="3">
         <v>1</v>
       </c>
@@ -1172,7 +1244,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1182,9 +1254,15 @@
       <c r="C7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="D7" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F7" s="3">
+        <v>2</v>
+      </c>
       <c r="G7" s="3">
         <v>-1</v>
       </c>
@@ -1197,7 +1275,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1207,11 +1285,15 @@
       <c r="C8" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E8" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F8" s="3"/>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
       <c r="G8" s="3">
         <v>1</v>
       </c>
@@ -1224,7 +1306,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1234,11 +1316,15 @@
       <c r="C9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E9" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F9" s="3"/>
+      <c r="F9" s="3">
+        <v>1</v>
+      </c>
       <c r="G9" s="3">
         <v>1</v>
       </c>
@@ -1251,7 +1337,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1261,11 +1347,15 @@
       <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E10" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F10" s="3"/>
+      <c r="F10" s="3">
+        <v>1</v>
+      </c>
       <c r="G10" s="3">
         <v>1</v>
       </c>
@@ -1288,12 +1378,22 @@
       <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F11" s="3">
+        <v>1</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="I11" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
@@ -1311,11 +1411,21 @@
       <c r="C12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F12" s="3">
+        <v>3</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>184</v>
+      </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -1334,13 +1444,21 @@
       <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F13" s="3">
+        <v>1</v>
+      </c>
       <c r="G13" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="H13" s="3"/>
+      <c r="H13" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
@@ -1349,7 +1467,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1359,12 +1477,18 @@
       <c r="C14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E14" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+      <c r="F14" s="3">
+        <v>2</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -1374,7 +1498,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1384,11 +1508,15 @@
       <c r="C15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E15" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="3">
+        <v>1</v>
+      </c>
       <c r="G15" s="3">
         <v>1</v>
       </c>
@@ -1401,7 +1529,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1411,11 +1539,15 @@
       <c r="C16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E16" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F16" s="3"/>
+      <c r="F16" s="3">
+        <v>1</v>
+      </c>
       <c r="G16" s="3">
         <v>1</v>
       </c>
@@ -1438,14 +1570,22 @@
       <c r="C17" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F17" s="3">
+        <v>3</v>
+      </c>
       <c r="G17" s="3" t="s">
         <v>176</v>
       </c>
       <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
+      <c r="I17" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
@@ -1463,15 +1603,27 @@
       <c r="C18" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F18" s="3">
+        <v>1</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+      <c r="K18" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="M18" s="4" t="s">
         <v>18</v>
       </c>
@@ -1486,15 +1638,27 @@
       <c r="C19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F19" s="3">
+        <v>1</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
+      <c r="K19" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="M19" s="4" t="s">
         <v>15</v>
       </c>
@@ -1509,20 +1673,32 @@
       <c r="C20" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F20" s="3">
+        <v>1</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0</v>
+      </c>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
+      <c r="K20" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="M20" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1532,12 +1708,18 @@
       <c r="C21" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E21" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
+      <c r="F21" s="3">
+        <v>2</v>
+      </c>
+      <c r="G21" s="3">
+        <v>-1</v>
+      </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1557,17 +1739,23 @@
       <c r="C22" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E22" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F22" s="3"/>
+      <c r="F22" s="3">
+        <v>2</v>
+      </c>
       <c r="G22" s="3">
         <v>-1</v>
       </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
+      <c r="J22" s="3" t="b">
+        <v>1</v>
+      </c>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="4" t="s">
@@ -1584,15 +1772,21 @@
       <c r="C23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E23" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F23" s="3"/>
+      <c r="F23" s="3">
+        <v>1</v>
+      </c>
       <c r="G23" s="3">
         <v>1</v>
       </c>
-      <c r="H23" s="3"/>
+      <c r="H23" s="3" t="s">
+        <v>186</v>
+      </c>
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
@@ -1611,11 +1805,15 @@
       <c r="C24" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D24" s="3"/>
+      <c r="D24" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E24" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F24" s="3"/>
+      <c r="F24" s="3">
+        <v>1</v>
+      </c>
       <c r="G24" s="3">
         <v>1</v>
       </c>
@@ -1638,15 +1836,29 @@
       <c r="C25" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
+      <c r="D25" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F25" s="3">
+        <v>1</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
+      <c r="I25" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
+      <c r="K25" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="M25" s="4" t="s">
         <v>15</v>
       </c>
@@ -1661,12 +1873,24 @@
       <c r="C26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
+      <c r="D26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F26" s="3">
+        <v>3</v>
+      </c>
+      <c r="G26" s="3">
+        <v>-1</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>183</v>
+      </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
@@ -1674,7 +1898,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1684,11 +1908,15 @@
       <c r="C27" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D27" s="3"/>
+      <c r="D27" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E27" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F27" s="3"/>
+      <c r="F27" s="3">
+        <v>1</v>
+      </c>
       <c r="G27" s="3">
         <v>1</v>
       </c>
@@ -1711,15 +1939,27 @@
       <c r="C28" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
+      <c r="D28" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" s="3">
+        <v>1</v>
+      </c>
+      <c r="G28" s="3">
+        <v>0</v>
+      </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
+      <c r="K28" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="M28" s="4" t="s">
         <v>15</v>
       </c>
@@ -1734,11 +1974,15 @@
       <c r="C29" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D29" s="3"/>
+      <c r="D29" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E29" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F29" s="3"/>
+      <c r="F29" s="3">
+        <v>1</v>
+      </c>
       <c r="G29" s="3">
         <v>1</v>
       </c>
@@ -1761,16 +2005,24 @@
       <c r="C30" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D30" s="3"/>
+      <c r="D30" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E30" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F30" s="3"/>
+      <c r="F30" s="3">
+        <v>3</v>
+      </c>
       <c r="G30" s="3">
         <v>-1</v>
       </c>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
+      <c r="H30" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>180</v>
+      </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
@@ -1788,12 +2040,18 @@
       <c r="C31" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D31" s="3"/>
+      <c r="D31" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E31" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
+      <c r="F31" s="3">
+        <v>3</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>177</v>
+      </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
       <c r="J31" s="3"/>
@@ -1803,7 +2061,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1813,16 +2071,24 @@
       <c r="C32" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+      <c r="D32" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F32" s="3">
+        <v>2</v>
+      </c>
       <c r="G32" s="3">
         <v>-1</v>
       </c>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
       <c r="J32" s="3"/>
-      <c r="K32" s="3"/>
+      <c r="K32" s="3" t="b">
+        <v>1</v>
+      </c>
       <c r="L32" s="3"/>
       <c r="M32" s="4" t="s">
         <v>15</v>
@@ -1838,11 +2104,21 @@
       <c r="C33" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+      <c r="D33" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F33" s="3">
+        <v>4</v>
+      </c>
+      <c r="G33" s="3">
+        <v>-1</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>189</v>
+      </c>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
@@ -1851,7 +2127,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -1861,15 +2137,21 @@
       <c r="C34" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D34" s="3"/>
+      <c r="D34" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E34" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F34" s="3"/>
+      <c r="F34" s="3">
+        <v>3</v>
+      </c>
       <c r="G34" s="3">
         <v>-1</v>
       </c>
-      <c r="H34" s="3"/>
+      <c r="H34" s="3" t="s">
+        <v>190</v>
+      </c>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
@@ -1888,20 +2170,32 @@
       <c r="C35" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
+      <c r="D35" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F35" s="3">
+        <v>1</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
       <c r="J35" s="3"/>
-      <c r="K35" s="3"/>
-      <c r="L35" s="3"/>
+      <c r="K35" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="M35" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -1911,11 +2205,15 @@
       <c r="C36" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D36" s="3"/>
+      <c r="D36" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E36" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F36" s="3"/>
+      <c r="F36" s="3">
+        <v>1</v>
+      </c>
       <c r="G36" s="3">
         <v>1</v>
       </c>
@@ -1928,7 +2226,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -1938,11 +2236,15 @@
       <c r="C37" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D37" s="3"/>
+      <c r="D37" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E37" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F37" s="3"/>
+      <c r="F37" s="3">
+        <v>1</v>
+      </c>
       <c r="G37" s="3">
         <v>1</v>
       </c>
@@ -1955,7 +2257,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -1965,11 +2267,15 @@
       <c r="C38" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D38" s="3"/>
+      <c r="D38" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E38" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F38" s="3"/>
+      <c r="F38" s="3">
+        <v>1</v>
+      </c>
       <c r="G38" s="3">
         <v>1</v>
       </c>
@@ -1982,7 +2288,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -1992,14 +2298,22 @@
       <c r="C39" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D39" s="3"/>
+      <c r="D39" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="E39" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
+      <c r="F39" s="3">
+        <v>4</v>
+      </c>
+      <c r="G39" s="3">
+        <v>-1</v>
+      </c>
       <c r="H39" s="3"/>
-      <c r="I39" s="3"/>
+      <c r="I39" s="3" t="s">
+        <v>181</v>
+      </c>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
@@ -2007,7 +2321,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2017,11 +2331,15 @@
       <c r="C40" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="3"/>
+      <c r="D40" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E40" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F40" s="3"/>
+      <c r="F40" s="3">
+        <v>1</v>
+      </c>
       <c r="G40" s="3">
         <v>1</v>
       </c>
@@ -2034,7 +2352,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -2044,11 +2362,15 @@
       <c r="C41" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D41" s="3"/>
+      <c r="D41" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E41" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F41" s="3"/>
+      <c r="F41" s="3">
+        <v>1</v>
+      </c>
       <c r="G41" s="3">
         <v>1</v>
       </c>
@@ -2061,7 +2383,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2071,11 +2393,15 @@
       <c r="C42" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D42" s="3"/>
+      <c r="D42" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E42" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="F42" s="3"/>
+        <v>149</v>
+      </c>
+      <c r="F42" s="3">
+        <v>3</v>
+      </c>
       <c r="G42" s="3" t="s">
         <v>176</v>
       </c>
@@ -2088,7 +2414,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2098,9 +2424,15 @@
       <c r="C43" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-      <c r="F43" s="3"/>
+      <c r="D43" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F43" s="3">
+        <v>2</v>
+      </c>
       <c r="G43" s="3">
         <v>-1</v>
       </c>
@@ -2113,7 +2445,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2123,16 +2455,22 @@
       <c r="C44" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D44" s="3"/>
+      <c r="D44" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="E44" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F44" s="3"/>
+      <c r="F44" s="3">
+        <v>3</v>
+      </c>
       <c r="G44" s="3">
         <v>-1</v>
       </c>
       <c r="H44" s="3"/>
-      <c r="I44" s="3"/>
+      <c r="I44" s="3" t="s">
+        <v>182</v>
+      </c>
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
@@ -2140,7 +2478,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2150,11 +2488,15 @@
       <c r="C45" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D45" s="3"/>
+      <c r="D45" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E45" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F45" s="3"/>
+      <c r="F45" s="3">
+        <v>1</v>
+      </c>
       <c r="G45" s="3">
         <v>1</v>
       </c>
@@ -2167,7 +2509,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2177,12 +2519,18 @@
       <c r="C46" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D46" s="3"/>
+      <c r="D46" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="E46" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
+      <c r="F46" s="3">
+        <v>3</v>
+      </c>
+      <c r="G46" s="3">
+        <v>-1</v>
+      </c>
       <c r="H46" s="3"/>
       <c r="I46" s="3"/>
       <c r="J46" s="3"/>
@@ -2192,7 +2540,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2202,11 +2550,15 @@
       <c r="C47" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D47" s="3"/>
+      <c r="D47" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E47" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F47" s="3"/>
+      <c r="F47" s="3">
+        <v>3</v>
+      </c>
       <c r="G47" s="3">
         <v>-1</v>
       </c>
@@ -2219,7 +2571,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2229,14 +2581,22 @@
       <c r="C48" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D48" s="3"/>
+      <c r="D48" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E48" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
+      <c r="F48" s="3">
+        <v>3</v>
+      </c>
+      <c r="G48" s="3">
+        <v>-1</v>
+      </c>
       <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
+      <c r="I48" s="3" t="s">
+        <v>179</v>
+      </c>
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
@@ -2244,7 +2604,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2254,14 +2614,22 @@
       <c r="C49" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D49" s="3"/>
+      <c r="D49" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="E49" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
+      <c r="F49" s="3">
+        <v>2</v>
+      </c>
+      <c r="G49" s="3">
+        <v>-1</v>
+      </c>
       <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
+      <c r="I49" s="3" t="s">
+        <v>183</v>
+      </c>
       <c r="J49" s="3"/>
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
@@ -2269,7 +2637,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="45" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" ht="45" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2279,11 +2647,15 @@
       <c r="C50" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="D50" s="3"/>
+      <c r="D50" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E50" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F50" s="3"/>
+      <c r="F50" s="3">
+        <v>1</v>
+      </c>
       <c r="G50" s="3">
         <v>1</v>
       </c>
@@ -2296,7 +2668,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="60" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" ht="60" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2306,11 +2678,15 @@
       <c r="C51" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="D51" s="3"/>
+      <c r="D51" s="3" t="s">
+        <v>141</v>
+      </c>
       <c r="E51" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F51" s="3"/>
+      <c r="F51" s="3">
+        <v>1</v>
+      </c>
       <c r="G51" s="3">
         <v>1</v>
       </c>
@@ -2324,14 +2700,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M51" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters blank="1"/>
-    </filterColumn>
-    <filterColumn colId="6">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M51" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not allowed" error="Pick from the list." promptTitle="topic" prompt="topic: main product area (see Definitions tab)" sqref="D2:D51" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"access,usability,playback,downloads,catalog,billing,support,other"</formula1>
@@ -2345,10 +2714,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not allowed" error="Pick from the list." promptTitle="sentiment" prompt="sentiment: -1 very negative to 1 very positive" sqref="G2:G51" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"-1,-0.5,0,0.5,1"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not allowed" error="Pick from the list." promptTitle="needs_review" prompt="needs_review: TRUE if context is missing to judge" sqref="J2:J51" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not allowed" error="Pick from the list." promptTitle="needs_review" prompt="needs_review: TRUE if context is missing to judge" sqref="J2:J17 J21:J24 J26:J27 J29:J34 J36:J51" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"FALSE,TRUE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not allowed" error="Pick from the list." promptTitle="ambiguous" prompt="ambiguous: TRUE if two labels are equally defensible" sqref="K2:K51" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not allowed" error="Pick from the list." promptTitle="ambiguous" prompt="ambiguous: TRUE if two labels are equally defensible" sqref="J35:K35 J18:J20 J25:K25 J28:K28 K2:K24 K26:K27 K29:K34 K36:K51" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"FALSE,TRUE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>